<commit_message>
fix: unify welding lab weights to DTE set
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EYF8ZViZ52j72cGLCGYpbD
</commit_message>
<xml_diff>
--- a/data/xlsx/aeosib--welding-and-fabrication-1g-2g-and-3g.xlsx
+++ b/data/xlsx/aeosib--welding-and-fabrication-1g-2g-and-3g.xlsx
@@ -702,7 +702,7 @@
         <v>0</v>
       </c>
       <c r="E19" s="27" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F19" s="27">
         <f>IFERROR(MIN(C19,D19)*E19/C19,0)</f>
@@ -726,7 +726,7 @@
         <v>0</v>
       </c>
       <c r="E20" s="27" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F20" s="27">
         <f>IFERROR(MIN(C20,D20)*E20/C20,0)</f>
@@ -846,7 +846,7 @@
         <v>0</v>
       </c>
       <c r="E25" s="27" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F25" s="27">
         <f>IFERROR(MIN(C25,D25)*E25/C25,0)</f>
@@ -918,7 +918,7 @@
         <v>0</v>
       </c>
       <c r="E28" s="27" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F28" s="27">
         <f>IFERROR(MIN(C28,D28)*E28/C28,0)</f>
@@ -942,7 +942,7 @@
         <v>0</v>
       </c>
       <c r="E29" s="27" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F29" s="27">
         <f>IFERROR(MIN(C29,D29)*E29/C29,0)</f>
@@ -966,7 +966,7 @@
         <v>0</v>
       </c>
       <c r="E30" s="27" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F30" s="27">
         <f>IFERROR(MIN(C30,D30)*E30/C30,0)</f>
@@ -990,7 +990,7 @@
         <v>0</v>
       </c>
       <c r="E31" s="27" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F31" s="27">
         <f>IFERROR(MIN(C31,D31)*E31/C31,0)</f>

</xml_diff>